<commit_message>
Update importer and styling
Automated migration updates generated by Experience Modernization Agent.

Changed files (8):
- tools/importer/import-ai-solutions-page.bundle.js
- tools/importer/import-customer-story-page.bundle.js
- tools/importer/reports/en-us/lp/dt/customer-stories-mclaren-racing.report.json
- tools/importer/reports/en-us/shop/scc/sc/artificial-intelligence.report.json
- tools/importer/reports/import-ai-solutions-page.report.xlsx
- tools/importer/reports/import-customer-story-page.report.xlsx
- tools/importer/reports/original-ai-bundle.report.xlsx
- tools/importer/transformers/dell-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-customer-story-page.report.xlsx
+++ b/tools/importer/reports/import-customer-story-page.report.xlsx
@@ -52,7 +52,7 @@
     <t>customer-story-page</t>
   </si>
   <si>
-    <t>2026-03-16T11:54:49.690Z</t>
+    <t>2026-03-16T12:29:34.829Z</t>
   </si>
   <si>
     <t>McLaren Formula 1® Team | Dell USA</t>
@@ -73,7 +73,7 @@
     <t>ai-solutions-page</t>
   </si>
   <si>
-    <t>2026-03-12T19:57:22.926Z</t>
+    <t>2026-03-16T12:28:46.522Z</t>
   </si>
   <si>
     <t>Artificial Intelligence Solutions | Dell USA</t>

</xml_diff>